<commit_message>
Quitar selectedName del Dashboard
</commit_message>
<xml_diff>
--- a/BASE.xlsx
+++ b/BASE.xlsx
@@ -1120,10 +1120,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0B2FADA4-9893-4AC8-B08B-1B38772D9F67}" name="Tabla1" displayName="Tabla1" ref="A1:D20" totalsRowShown="0">
   <autoFilter ref="A1:D20" xr:uid="{0B2FADA4-9893-4AC8-B08B-1B38772D9F67}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{F0672D35-EF69-417C-8B8C-66C978009A5D}" name="CARGO" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{5975F1B4-DF2B-463F-8972-02D223F86D36}" name="NOMBRE" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{F2A051C8-1DB2-477D-9151-6FDCC287C8F6}" name="CORREO" dataDxfId="13" dataCellStyle="Hipervínculo"/>
-    <tableColumn id="4" xr3:uid="{24EC387A-C737-4F86-A384-D8F2D8869E17}" name="CONTRASEÑA" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{F0672D35-EF69-417C-8B8C-66C978009A5D}" name="CARGO" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{5975F1B4-DF2B-463F-8972-02D223F86D36}" name="NOMBRE" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F2A051C8-1DB2-477D-9151-6FDCC287C8F6}" name="CORREO" dataDxfId="9" dataCellStyle="Hipervínculo"/>
+    <tableColumn id="4" xr3:uid="{24EC387A-C737-4F86-A384-D8F2D8869E17}" name="CONTRASEÑA" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1133,10 +1133,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BA22E976-A805-456E-8106-00B533F961C0}" name="Tabla13" displayName="Tabla13" ref="A1:D21" totalsRowShown="0">
   <autoFilter ref="A1:D21" xr:uid="{BA22E976-A805-456E-8106-00B533F961C0}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{11EE423A-76B8-46A6-9836-923C6840DB45}" name="CARGO" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{50C3DC64-9186-418F-960B-04B66E8CCF85}" name="NOMBRE" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{9A23C464-6E28-4CAB-8120-17352AF47B66}" name="CORREO" dataDxfId="9" dataCellStyle="Hipervínculo"/>
-    <tableColumn id="4" xr3:uid="{7F0CA33E-B8DF-4486-9487-9490402C11A3}" name="CONTRASEÑA" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{11EE423A-76B8-46A6-9836-923C6840DB45}" name="CARGO" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{50C3DC64-9186-418F-960B-04B66E8CCF85}" name="NOMBRE" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{9A23C464-6E28-4CAB-8120-17352AF47B66}" name="CORREO" dataDxfId="13" dataCellStyle="Hipervínculo"/>
+    <tableColumn id="4" xr3:uid="{7F0CA33E-B8DF-4486-9487-9490402C11A3}" name="CONTRASEÑA" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Mejoras: Luisa restringida, reconocimientos, WhatsApp, estados RS con colores, historial visible, umbrales 6/2/1 mes
</commit_message>
<xml_diff>
--- a/BASE.xlsx
+++ b/BASE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrea Huamani\Documents\app-retroalimentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E24BF40F-5A6A-491B-A317-2582EB4E6518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BB49C12-53F0-4C28-A006-01157E42BB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8ACB5D83-9E92-435F-BD98-53BFD5220FF2}"/>
   </bookViews>
@@ -20,6 +20,7 @@
     <sheet name="FUNCIONES" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="266">
   <si>
     <t>Gerente(a) General</t>
   </si>
@@ -822,14 +823,32 @@
     <t>%</t>
   </si>
   <si>
-    <t>FALTA MILAGROS FLORES</t>
+    <t>lrocca@ferco-medical.com</t>
+  </si>
+  <si>
+    <t>Analista de DT</t>
+  </si>
+  <si>
+    <t>WSP</t>
+  </si>
+  <si>
+    <t>MARIA QUIQUIA</t>
+  </si>
+  <si>
+    <t>mquiquia@ferco-medical.com</t>
+  </si>
+  <si>
+    <t>ENCARGADO DE COORDINACION</t>
+  </si>
+  <si>
+    <t>Manuel Jimenez</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -877,8 +896,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -921,6 +956,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -950,7 +991,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -995,9 +1036,24 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1130,13 +1186,17 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BA22E976-A805-456E-8106-00B533F961C0}" name="Tabla13" displayName="Tabla13" ref="A1:D21" totalsRowShown="0">
-  <autoFilter ref="A1:D21" xr:uid="{BA22E976-A805-456E-8106-00B533F961C0}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BA22E976-A805-456E-8106-00B533F961C0}" name="Tabla13" displayName="Tabla13" ref="A1:E22" totalsRowShown="0">
+  <autoFilter ref="A1:E22" xr:uid="{BA22E976-A805-456E-8106-00B533F961C0}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E22">
+    <sortCondition ref="B1:B22"/>
+  </sortState>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{11EE423A-76B8-46A6-9836-923C6840DB45}" name="CARGO" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{50C3DC64-9186-418F-960B-04B66E8CCF85}" name="NOMBRE" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{9A23C464-6E28-4CAB-8120-17352AF47B66}" name="CORREO" dataDxfId="13" dataCellStyle="Hipervínculo"/>
     <tableColumn id="4" xr3:uid="{7F0CA33E-B8DF-4486-9487-9490402C11A3}" name="CONTRASEÑA" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{ED19BDD6-6D51-4DF5-B3F7-F0DE4BBE6BCD}" name="WSP"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1796,7 +1856,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E53526D9-56E6-464E-97EA-0ED2E02033E1}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.109375" bestFit="1" customWidth="1"/>
@@ -1805,7 +1865,7 @@
     <col min="4" max="4" width="17" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>166</v>
       </c>
@@ -1818,306 +1878,389 @@
       <c r="D1" s="11" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>180</v>
+        <v>37</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>146</v>
+        <v>41</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>183</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="18">
+        <v>905471351</v>
+      </c>
+      <c r="I3" s="17"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>178</v>
+        <v>108</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>59</v>
+        <v>116</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>177</v>
+      <c r="E4" s="18">
+        <v>983706298</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5" s="18">
+        <v>957657709</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>119</v>
+        <v>180</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>158</v>
+        <v>67</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>146</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" s="18">
+        <v>912390793</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>137</v>
+        <v>23</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="18">
+        <v>933537891</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>108</v>
+        <v>35</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>135</v>
+        <v>36</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="18">
+        <v>967246293</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>108</v>
+        <v>181</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>116</v>
+        <v>83</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" s="18">
+        <v>961553827</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>102</v>
+        <v>6</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" s="18">
+        <v>975441208</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" s="18">
+        <v>955682681</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12" s="18">
+        <v>970673750</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>182</v>
+        <v>260</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>154</v>
+        <v>97</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>259</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>172</v>
+        <v>119</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>23</v>
+        <v>265</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>171</v>
+      <c r="E14" s="18">
+        <v>912390773</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>177</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E15" s="18">
+        <v>945839491</v>
+      </c>
+      <c r="F15" s="18"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="19" t="s">
+        <v>264</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>263</v>
+      </c>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23">
+        <v>958130958</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>6</v>
+        <v>135</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" s="18">
+        <v>995890071</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" s="18">
+        <v>990800119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>168</v>
-      </c>
-      <c r="D19" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="D19" s="16" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" s="18">
+        <v>999304625</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>37</v>
+        <v>179</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>183</v>
+        <v>147</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="16" t="s">
-        <v>259</v>
-      </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="12"/>
+      <c r="E20" s="18">
+        <v>977910077</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E21" s="18">
+        <v>908858199</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="18">
+        <v>924550094</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{F0CD9141-6B79-4947-8A86-831F3E1D0646}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{BE59AA90-8270-4D29-92F3-4A3C71C61537}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{E0A5591B-0704-4AE3-91C4-95B77514C40F}"/>
-    <hyperlink ref="C17" r:id="rId4" xr:uid="{05D178B4-0DC9-4922-BF0D-1AD19E6D6970}"/>
-    <hyperlink ref="C16" r:id="rId5" xr:uid="{1A3176D9-AB72-4CC1-A591-8967390C112C}"/>
-    <hyperlink ref="C11" r:id="rId6" xr:uid="{27ABDC03-0BD4-4A8F-AD3A-9FCD9DFD900E}"/>
-    <hyperlink ref="C15" r:id="rId7" xr:uid="{8C5D6C8F-B50A-4852-9C02-BBEA4AFA4298}"/>
-    <hyperlink ref="C14" r:id="rId8" xr:uid="{70EF91E9-4672-4316-AB1E-7AE2C61BB215}"/>
-    <hyperlink ref="C13" r:id="rId9" xr:uid="{5B866A9F-8550-4CE8-B6B2-C31579C06497}"/>
-    <hyperlink ref="C12" r:id="rId10" xr:uid="{9AE13416-345C-4B60-BB59-B331849072A2}"/>
-    <hyperlink ref="C10" r:id="rId11" xr:uid="{4112AC9B-08C8-4C8C-B08F-33DE0E550DD2}"/>
-    <hyperlink ref="C9" r:id="rId12" xr:uid="{88F87024-2C68-4AB3-86C2-71C9AA7CCDB5}"/>
-    <hyperlink ref="C6" r:id="rId13" xr:uid="{74D55FFF-B8B8-4125-A004-8CE75EF7E80C}"/>
-    <hyperlink ref="C5" r:id="rId14" xr:uid="{CC95F048-72C1-4F9E-BC43-D87C97D61646}"/>
-    <hyperlink ref="C8" r:id="rId15" xr:uid="{0D1819B8-BC1B-4ABE-BEE0-BF3B91209A07}"/>
-    <hyperlink ref="C7" r:id="rId16" xr:uid="{2D939BD9-B992-4986-919D-2DF2DDB6F093}"/>
-    <hyperlink ref="C18" r:id="rId17" xr:uid="{8BEC1B05-22C3-42B0-AD9B-1A4F6D40D679}"/>
-    <hyperlink ref="C19" r:id="rId18" xr:uid="{86ED3AB2-9973-45D4-93F2-175D13298D32}"/>
-    <hyperlink ref="C20" r:id="rId19" xr:uid="{B79150EE-27A7-4F3D-8D4E-BC636A2C15CB}"/>
+    <hyperlink ref="C6" r:id="rId1" xr:uid="{F0CD9141-6B79-4947-8A86-831F3E1D0646}"/>
+    <hyperlink ref="C20" r:id="rId2" xr:uid="{BE59AA90-8270-4D29-92F3-4A3C71C61537}"/>
+    <hyperlink ref="C18" r:id="rId3" xr:uid="{E0A5591B-0704-4AE3-91C4-95B77514C40F}"/>
+    <hyperlink ref="C10" r:id="rId4" xr:uid="{05D178B4-0DC9-4922-BF0D-1AD19E6D6970}"/>
+    <hyperlink ref="C8" r:id="rId5" xr:uid="{1A3176D9-AB72-4CC1-A591-8967390C112C}"/>
+    <hyperlink ref="C12" r:id="rId6" xr:uid="{27ABDC03-0BD4-4A8F-AD3A-9FCD9DFD900E}"/>
+    <hyperlink ref="C21" r:id="rId7" xr:uid="{8C5D6C8F-B50A-4852-9C02-BBEA4AFA4298}"/>
+    <hyperlink ref="C7" r:id="rId8" xr:uid="{70EF91E9-4672-4316-AB1E-7AE2C61BB215}"/>
+    <hyperlink ref="C11" r:id="rId9" xr:uid="{5B866A9F-8550-4CE8-B6B2-C31579C06497}"/>
+    <hyperlink ref="C22" r:id="rId10" xr:uid="{9AE13416-345C-4B60-BB59-B331849072A2}"/>
+    <hyperlink ref="C3" r:id="rId11" xr:uid="{4112AC9B-08C8-4C8C-B08F-33DE0E550DD2}"/>
+    <hyperlink ref="C4" r:id="rId12" xr:uid="{88F87024-2C68-4AB3-86C2-71C9AA7CCDB5}"/>
+    <hyperlink ref="C14" r:id="rId13" xr:uid="{74D55FFF-B8B8-4125-A004-8CE75EF7E80C}"/>
+    <hyperlink ref="C15" r:id="rId14" xr:uid="{CC95F048-72C1-4F9E-BC43-D87C97D61646}"/>
+    <hyperlink ref="C17" r:id="rId15" xr:uid="{0D1819B8-BC1B-4ABE-BEE0-BF3B91209A07}"/>
+    <hyperlink ref="C5" r:id="rId16" xr:uid="{2D939BD9-B992-4986-919D-2DF2DDB6F093}"/>
+    <hyperlink ref="C19" r:id="rId17" xr:uid="{8BEC1B05-22C3-42B0-AD9B-1A4F6D40D679}"/>
+    <hyperlink ref="C9" r:id="rId18" xr:uid="{86ED3AB2-9973-45D4-93F2-175D13298D32}"/>
+    <hyperlink ref="C2" r:id="rId19" xr:uid="{B79150EE-27A7-4F3D-8D4E-BC636A2C15CB}"/>
+    <hyperlink ref="C13" r:id="rId20" xr:uid="{85CDCA01-8422-4C88-92C9-F1F3641636B7}"/>
+    <hyperlink ref="C16" r:id="rId21" xr:uid="{CDDB4FC1-4645-4D3D-9AA9-4D801AB4B822}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId20"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId22"/>
   <tableParts count="1">
-    <tablePart r:id="rId21"/>
+    <tablePart r:id="rId23"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>